<commit_message>
Alterações finais de BI e automação
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-01-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-01-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-01-2026 20:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-01-2026 20:16
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-01-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7698,7 +7698,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7884,7 +7884,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9930,7 +9930,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-01-2026 20:41
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9558,7 +9558,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10116,7 +10116,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15634,7 +15634,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-01-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-01-2026 20:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 31-01-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-02-2026 20:27
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-02-2026 20:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-02-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-02-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-02-2026 20:25
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-02-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-02-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-02-2026 20:28
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-02-2026 20:22
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-02-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-03-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-03-2026 20:30
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-03-2026 20:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-03-2026 20:32
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-03-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-03-2026 20:25
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-03-2026 20:25
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 14-03-2026 20:19
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 15-03-2026 20:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-03-2026 20:32
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-03-2026 20:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-03-2026 20:19
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-03-2026 20:33
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-03-2026 20:34
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-03-2026 20:30
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-03-2026 20:30
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 28-03-2026 20:21
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-03-2026 20:38
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-04-2026 20:28
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-04-2026 20:28
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-04-2026 20:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-04-2026 20:32
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-04-2026 20:27
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-04-2026 20:38
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-04-2026 20:28
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-04-2026 20:29
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-04-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 29-04-2026 20:54
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-04-2026 20:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-05-2026 20:44
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-05-2026 21:00
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-05-2026 20:49
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 16-05-2026 20:41
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 21-05-2026 21:25
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-05-2026 21:06
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 23-05-2026 20:43
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-05-2026 20:45
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-05-2026 21:02
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-05-2026 21:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 31-05-2026 20:51
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-06-2026 22:21
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 03-06-2026 22:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-06-2026 21:03
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-06-2026 21:36
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-06-2026 21:33
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-06-2026 21:54
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-06-2026 21:28
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-06-2026 21:05
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 18-06-2026 22:00
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-06-2026 21:05
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-06-2026 21:07
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 22-06-2026 21:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 25-06-2026 21:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 26-06-2026 21:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-06-2026 20:53
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 01-07-2026 21:20
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-07-2026 20:47
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-07-2026 20:50
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 06-07-2026 21:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-07-2026 20:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-07-2026 21:15
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-07-2026 21:03
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-07-2026 20:38
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-07-2026 20:52
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 20-07-2026 21:04
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 27-07-2026 21:05
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 30-07-2026 20:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 05-08-2026 20:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-08-2026 20:24
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-08-2026 20:35
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 13-08-2026 20:33
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 17-08-2026 20:18
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 19-08-2026 20:17
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 24-08-2026 20:22
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 31-08-2026 23:34
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 02-09-2026 22:10
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 04-09-2026 21:59
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 07-09-2026 22:26
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>filhote</t>
+          <t>puppy</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 08-09-2026 22:11
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 09-09-2026 22:09
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spot</t>
+          <t>spoton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 10-09-2026 22:07
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -9546,7 +9546,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10042,7 +10042,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>puppy</t>
+          <t>filhote</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 11-09-2026 22:09
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>transdermal</t>
+          <t>plus</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Coleta automática em 12-09-2026 21:51
</commit_message>
<xml_diff>
--- a/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
+++ b/Tratamento/src/Dados_limpos/novos/limpo_petlove_20250927_124701.xlsx
@@ -7686,7 +7686,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7872,7 +7872,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>plus</t>
+          <t>transdermal</t>
         </is>
       </c>
     </row>
@@ -9670,7 +9670,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9918,7 +9918,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>
@@ -9980,7 +9980,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>spoton</t>
+          <t>spot</t>
         </is>
       </c>
     </row>

</xml_diff>